<commit_message>
Homepage UI/UX: staging results (browser + Android/iOS app emulation), split check
Guest suite on test.gokesari.com after it built #214 + #215 + #218:
browser 30/30 (1 skipped), Android app 20/20, iOS app 22/22 cases;
batch-2026-10-remote + branding-footer 20/20; Lighthouse mobile 88 / 96,
accessibility 100. Both sites on the split layout (switch-status).
DEF-13 closed with its root cause (Hostinger's SELLER_DATABASE_URL, #218).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gs4EQHD7GwAULfSqxrdL9g
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GoKesari_Homepage_UIUX_Status_2026-10-20.xlsx
+++ b/docs/gokesari-audit/GoKesari_Homepage_UIUX_Status_2026-10-20.xlsx
@@ -17,13 +17,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Features'!$A$1:$K$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flows'!$A$1:$K$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Cases'!$A$1:$L$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Defects'!$A$1:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lighthouse'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$D$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lighthouse'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$D$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -614,284 +614,284 @@
           <t>Playwright pass rate — Staging</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>30/30 (100%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Playwright pass rate — Production</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+          <t xml:space="preserve">  run used for Staging</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test.gokesari.com (https://test.gokesari.com, 2026-10-20T05:51)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Playwright pass rate — Android</t>
+          <t>Playwright pass rate — Production</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>20/20 (100%)</t>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  run used for Android</t>
+          <t>Playwright pass rate — Android</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>localhost_3000-app-android (http://localhost:3000, 2026-10-19T22:06)</t>
+          <t>20/20 (100%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Playwright pass rate — iOS</t>
+          <t xml:space="preserve">  run used for Android</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>22/22 (100%)</t>
+          <t>test.gokesari.com-app-android (https://test.gokesari.com, 2026-10-20T05:54)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  run used for iOS</t>
+          <t>Playwright pass rate — iOS</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>localhost_3000-app-ios (http://localhost:3000, 2026-10-19T22:06)</t>
+          <t>22/22 (100%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Unit + integration (Vitest, local, single DB)</t>
+          <t xml:space="preserve">  run used for iOS</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2,254 / 2,255 first run; the 1 failure (SEC-03) was a BOOTSTRAP_ADMIN_EMAILS value in the local .env; re-run of that file 28/28 → effectively 2,255 / 2,255</t>
+          <t>test.gokesari.com-app-ios (https://test.gokesari.com, 2026-10-20T05:56)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>New tests on the split layout (local)</t>
+          <t>Unit + integration (Vitest, local, single DB)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>39 / 39 (homepage-uiux unit + integration, price-comparison, db-split ownership); migrations 0086 → core, 0087 → seller applied on an existing split layout</t>
+          <t>2,254 / 2,255 first run; the 1 failure (SEC-03) was a BOOTSTRAP_ADMIN_EMAILS value in the local .env; re-run of that file 28/28 → effectively 2,255 / 2,255</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mobile app (mobile/)</t>
+          <t>New tests on the split layout (local)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>typecheck ✓, lint ✓, 36 / 36 tests, Expo bundles Android + iOS ✓</t>
+          <t>39 / 39 (homepage-uiux unit + integration, price-comparison, db-split ownership); migrations 0086 → core, 0087 → seller applied on an existing split layout</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Lint / typecheck (web)</t>
+          <t>Mobile app (mobile/)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>0 errors (4 pre-existing warnings), tsc clean, production build ✓</t>
+          <t>typecheck ✓, lint ✓, 36 / 36 tests, Expo bundles Android + iOS ✓</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Android APK 1.3.0 (GitHub 'Android APK' workflow, PR #214)</t>
+          <t>Lint / typecheck (web)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Built ✓ — artifacts GoKesari-preview-apk and GoKesari-production-apk (run 39333658232, expire 18 Nov 2026)</t>
+          <t>0 errors (4 pre-existing warnings), tsc clean, production build ✓</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CI on PR #214</t>
+          <t>Android APK 1.3.0 (GitHub 'Android APK' workflow, PR #214)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>scope ✓, test ✓ (full suite), test-split ✓ (two-database layout), mobile ✓, APK preview ✓, APK production ✓ — merged into staging 19 Oct 22:49 UTC</t>
+          <t>Built ✓ — artifacts GoKesari-preview-apk and GoKesari-production-apk (run 39333658232, expire 18 Nov 2026)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Existing E2E regression (local)</t>
+          <t>CI on PR #214</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>acceptance 5/5 (sign-in, wallet top-up, subscribe 2 L/day, daily order + charge, change tomorrow, offline-only, access control, cron auth); mobile-app 5/7 (2 need the dev sign-in form, run on the dev server); branding-footer 8/8 (updated to the new footer); inventory-accounting, document-browser-read pass on the production build; regression-items-a-e 10 pass, then stops at the stale C1 step (Seller Central moved the shop contact card on 14 Oct — predates this change; later serial steps not reached, covered by integration tests)</t>
+          <t>scope ✓, test ✓ (full suite), test-split ✓ (two-database layout), mobile ✓, APK preview ✓, APK production ✓ — merged into staging 19 Oct 22:49 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — PR #214 merged</t>
+          <t>Existing E2E regression (local)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>19 Oct 2026 22:49 UTC (merge 1f4cd76)</t>
+          <t>acceptance 5/5 (sign-in, wallet top-up, subscribe 2 L/day, daily order + charge, change tomorrow, offline-only, access control, cron auth); mobile-app 5/7 (2 need the dev sign-in form, run on the dev server); branding-footer 8/8 (updated to the new footer); inventory-accounting, document-browser-read pass on the production build; regression-items-a-e 10 pass, then stops at the stale C1 step (Seller Central moved the shop contact card on 14 Oct — predates this change; later serial steps not reached, covered by integration tests)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — first build</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-00, fixed by #215) — then not rebuilt by Hostinger (DEF-13)</t>
+          <t>Staging remote regression (batch-2026-10-remote + branding-footer)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>20 / 20 passed on test.gokesari.com (20 Oct 05:58 UTC)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — fix PR #215 merged</t>
+          <t>Deploy — Staging — PR #214 merged</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>19 Oct 2026 23:50 UTC (merge e6dab2d)</t>
+          <t>19 Oct 2026 22:49 UTC (merge 1f4cd76)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging database (split: core + seller)</t>
+          <t>Deploy — Staging — fix PR #215 merged</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Test database workflow run 39344001502, 23:51 UTC: backup ✓, 0086 → core, 0087 → seller, verify newest 0087 ✓</t>
+          <t>19 Oct 2026 23:50 UTC (merge e6dab2d)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — site build after #215</t>
+          <t>Deploy — Staging database (split: core + seller)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Not live at 00:47 UTC 20 Oct (57 min after the merge); site still on the build of 19 Oct 21:15 UTC</t>
+          <t>Test database run 39344001502, 23:51 UTC: backup ✓, 0086 → core, 0087 → seller, verify newest 0087 ✓</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Production — database migrate (0086, 0087)</t>
+          <t>Deploy — Staging — site build</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Held until staging passes (prod-db.yml verify, run 39338789453: production lacks only 0086 and 0087)</t>
+          <t>20 Oct 04:47 UTC: staging c2b1018 (#214 + #215 + #218) after Hostinger's SELLER_DATABASE_URL was corrected (DEF-13)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Production — release staging → main</t>
+          <t>Deploy — Split layout — staging</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Held until staging passes</t>
+          <t>split: core neondb, seller gokesari_seller (Database split switch-status, run 39376681434, 05:46 UTC)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Open blockers</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>5</v>
+          <t>Deploy — Split layout — production</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>split: core neondb, seller PROD_SELLER_DATABASE_URL (Database split switch-status, run 39376683693, 05:46 UTC)</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Staging deploy: Hostinger has not rebuilt test.gokesari.com since 19 Oct 21:15 UTC, so the new home is not live there (DEF-13). Owner: check the build log in hPanel and redeploy ('Settings and redeploy'). Production (database migration, release, tests) waits for staging.</t>
+          <t>Deploy — Production database (0086, 0087)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Production database run 39372089225, 04:55 UTC: restore point, migrate, state after ✓</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>iOS native build: the 'iPhone app' workflow needs the repository secret EXPO_TOKEN and the Expo project id in mobile/app.config.ts (last run 18 Oct failed on both). Owner: add them (mobile/README.md 'iPhone builds from GitHub'), then Actions → iPhone app → Run (preview).</t>
+          <t>Deploy — Production — release #219 (staging → main)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>merged 20 Oct 05:39 UTC (80189e2), owner-approved</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Android emulator / iOS simulator: this cloud environment has no Android SDK / KVM and no macOS. App checks ran as Playwright emulation of the app WebView (app user agent, touch, phone widths); the Android APKs are built by the 'Android APK' workflow on the PR.</t>
-        </is>
+          <t>Open blockers</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -902,12 +902,36 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Signed-in flows on staging / production: remote sign-in needs an emailed one-time code from a mailbox this run cannot read; signed-in flows were run locally. Staging sandbox payment (Cashfree) needs a signed-in session → not run on staging in this pass.</t>
+          <t>iOS native build: the 'iPhone app' workflow needs the repository secret EXPO_TOKEN and the Expo project id in mobile/app.config.ts (last run 18 Oct failed on both). Owner: add them (mobile/README.md 'iPhone builds from GitHub'), then Actions → iPhone app → Run (preview).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Android emulator / iOS simulator: this cloud environment has no Android SDK / KVM and no macOS. App checks ran as Playwright emulation of the app WebView (app user agent, touch, phone widths); the Android APKs are built by the 'Android APK' workflow on the PR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Signed-in flows on staging / production: they need the emailed sign-in code of a test account. Reading it from the test mailbox was refused by this session's permission check (D-28); signed-in flows ran locally (F1-ACCOUNT-DESKTOP, F3-EMPTY-STATES, F6-FLOATING-CART, F2-RECENT-ACCOUNT, F1-BANNER-ADMIN). Staging sandbox payment (Cashfree) needs a signed-in session → not run in this pass.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B35"/>
+  <autoFilter ref="A1:B37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1022,14 +1046,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -1075,14 +1099,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -1132,14 +1156,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -1189,14 +1213,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -1242,14 +1266,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1295,14 +1319,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1352,14 +1376,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1409,14 +1433,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1462,14 +1486,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1515,14 +1539,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1568,14 +1592,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1621,14 +1645,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1678,14 +1702,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1731,14 +1755,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1784,14 +1808,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1837,14 +1861,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1890,14 +1914,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1943,14 +1967,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -2000,14 +2024,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -2053,14 +2077,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -2106,14 +2130,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -2159,14 +2183,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -2212,14 +2236,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2265,14 +2289,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2318,14 +2342,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -2375,14 +2399,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -2489,14 +2513,14 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2631,14 +2655,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -2684,14 +2708,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -2737,14 +2761,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -2790,14 +2814,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -2843,14 +2867,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2896,14 +2920,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -2949,14 +2973,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -3002,14 +3026,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -3055,14 +3079,14 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-13)</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (waits for staging)</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the gokesari.com build</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -3910,7 +3934,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/APP-VOICE-1.2.0.png</t>
+          <t>iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/APP-VOICE-1.2.0.png</t>
         </is>
       </c>
     </row>
@@ -3972,7 +3996,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/APP-VOICE-1.3.0.png</t>
+          <t>iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/APP-VOICE-1.3.0.png</t>
         </is>
       </c>
     </row>
@@ -4136,9 +4160,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -4159,8 +4183,9 @@
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F1-DRAWER-GUEST.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F1-DRAWER-GUEST.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F1-DRAWER-GUEST.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F1-DRAWER-GUEST.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F1-DRAWER-GUEST.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F1-DRAWER-GUEST.png</t>
         </is>
       </c>
     </row>
@@ -4200,9 +4225,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -4223,8 +4248,9 @@
       <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F1-HERO.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F1-HERO.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F1-HERO.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F1-HERO.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F1-HERO.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F1-HERO.png</t>
         </is>
       </c>
     </row>
@@ -4264,9 +4290,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -4384,9 +4410,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -4407,8 +4433,9 @@
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F2-SUGGEST-DESKTOP.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F2-SUGGEST-DESKTOP.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F2-SUGGEST-DESKTOP.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F2-SUGGEST-DESKTOP.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F2-SUGGEST-DESKTOP.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F2-SUGGEST-DESKTOP.png</t>
         </is>
       </c>
     </row>
@@ -4448,9 +4475,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -4471,8 +4498,9 @@
       <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F2-VOICE.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F2-VOICE.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F2-VOICE.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F2-VOICE.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F2-VOICE.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F2-VOICE.png</t>
         </is>
       </c>
     </row>
@@ -4574,9 +4602,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -4597,8 +4625,9 @@
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F3-SEARCH-EMPTY.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F3-SEARCH-EMPTY.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F3-SEARCH-EMPTY.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F3-SEARCH-EMPTY.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F3-SEARCH-EMPTY.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F3-SEARCH-EMPTY.png</t>
         </is>
       </c>
     </row>
@@ -4638,9 +4667,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -4661,8 +4690,9 @@
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F4-COMPARE.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F4-COMPARE.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F4-COMPARE.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F4-COMPARE.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F4-COMPARE.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F4-COMPARE.png</t>
         </is>
       </c>
     </row>
@@ -4702,9 +4732,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -4725,8 +4755,9 @@
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F5-FOOTER.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F5-FOOTER.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F5-FOOTER.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F5-FOOTER.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F5-FOOTER.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F5-FOOTER.png</t>
         </is>
       </c>
     </row>
@@ -4828,9 +4859,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -4851,8 +4882,9 @@
       <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F6-LOCATION-SHEET.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F6-LOCATION-SHEET.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F6-LOCATION-SHEET.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F6-LOCATION-SHEET.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F6-LOCATION-SHEET.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F6-LOCATION-SHEET.png</t>
         </is>
       </c>
     </row>
@@ -4892,9 +4924,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -4915,8 +4947,9 @@
       <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F6-STICKY.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/F6-STICKY.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/F6-STICKY.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F6-STICKY.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F6-STICKY.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F6-STICKY.png</t>
         </is>
       </c>
     </row>
@@ -4956,9 +4989,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -4978,7 +5011,8 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-en.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-en.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-en.png</t>
         </is>
       </c>
     </row>
@@ -5018,9 +5052,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -5040,7 +5074,8 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-hi.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-hi.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-hi.png</t>
         </is>
       </c>
     </row>
@@ -5080,9 +5115,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -5102,7 +5137,8 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-mr.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-mr.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-mr.png</t>
         </is>
       </c>
     </row>
@@ -5142,9 +5178,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -5164,7 +5200,8 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-en.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-en.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-en.png</t>
         </is>
       </c>
     </row>
@@ -5204,9 +5241,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -5226,7 +5263,8 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-hi.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-hi.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-hi.png</t>
         </is>
       </c>
     </row>
@@ -5266,9 +5304,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -5288,7 +5326,8 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-mr.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-mr.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-mr.png</t>
         </is>
       </c>
     </row>
@@ -5328,9 +5367,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -5351,8 +5390,9 @@
       <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-360-en.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-360-en.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-360-en.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-360-en.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-360-en.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-360-en.png</t>
         </is>
       </c>
     </row>
@@ -5392,9 +5432,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -5415,8 +5455,9 @@
       <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-360-hi.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-360-hi.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-360-hi.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-360-hi.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-360-hi.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-360-hi.png</t>
         </is>
       </c>
     </row>
@@ -5456,9 +5497,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -5479,8 +5520,9 @@
       <c r="L27" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-360-mr.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-360-mr.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-360-mr.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-360-mr.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-360-mr.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-360-mr.png</t>
         </is>
       </c>
     </row>
@@ -5520,9 +5562,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -5543,8 +5585,9 @@
       <c r="L28" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-390-en.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-390-en.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-390-en.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-390-en.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-390-en.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-390-en.png</t>
         </is>
       </c>
     </row>
@@ -5584,9 +5627,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -5607,8 +5650,9 @@
       <c r="L29" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-390-hi.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-390-hi.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-390-hi.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-390-hi.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-390-hi.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-390-hi.png</t>
         </is>
       </c>
     </row>
@@ -5648,9 +5692,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -5671,8 +5715,9 @@
       <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-390-mr.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-390-mr.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-390-mr.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-390-mr.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-390-mr.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-390-mr.png</t>
         </is>
       </c>
     </row>
@@ -5712,9 +5757,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -5735,8 +5780,9 @@
       <c r="L31" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-414-en.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-414-en.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-414-en.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-414-en.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-414-en.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-414-en.png</t>
         </is>
       </c>
     </row>
@@ -5776,9 +5822,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -5799,8 +5845,9 @@
       <c r="L32" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-414-hi.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-414-hi.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-414-hi.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-414-hi.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-414-hi.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-414-hi.png</t>
         </is>
       </c>
     </row>
@@ -5840,9 +5887,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -5863,8 +5910,9 @@
       <c r="L33" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-414-mr.png
-Android: e2e-evidence/homepage-uiux/localhost_3000-app-android/HP-414-mr.png
-iOS: e2e-evidence/homepage-uiux/localhost_3000-app-ios/HP-414-mr.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-414-mr.png
+Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-414-mr.png
+iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-414-mr.png</t>
         </is>
       </c>
     </row>
@@ -5904,9 +5952,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -5926,7 +5974,8 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-en.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-en.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-en.png</t>
         </is>
       </c>
     </row>
@@ -5966,9 +6015,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -5988,7 +6037,8 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-hi.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-hi.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-hi.png</t>
         </is>
       </c>
     </row>
@@ -6028,9 +6078,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -6050,7 +6100,8 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-mr.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-mr.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-mr.png</t>
         </is>
       </c>
     </row>
@@ -6090,9 +6141,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -6148,9 +6199,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -6170,7 +6221,8 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/REG-SITE-HEADER.png</t>
+          <t>Local: e2e-evidence/homepage-uiux/localhost_3000/REG-SITE-HEADER.png
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/REG-SITE-HEADER.png</t>
         </is>
       </c>
     </row>
@@ -6707,7 +6759,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>test.gokesari.com has not been rebuilt by Hostinger since 19 Oct 21:15 UTC (Last-Modified of its static files; build pDsNwMAZ6y75Yn2ns8gHO). The pushes to staging for #213 (22:24), #214 (22:49) and #215 (23:50) are not live: the site still serves the old home and /api/search/suggest answers 404 after 57 min of polling. The staging databases are already migrated (Test database run 39344001502), and the same migrator succeeded there with the real URLs.</t>
+          <t>test.gokesari.com did not build #213–#215 (19 Oct 22:24 → 20 Oct 04:45 UTC): Hostinger's build stopped in migrate-on-build. Root cause (found from the Hostinger build log, PR #218): the test site's SELLER_DATABASE_URL opened a different database from the seller database the core's foreign tables read (its migration log ended at 0075), so the split migrator refused to go on. The test database itself was already migrated by the Test database workflow.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -6722,12 +6774,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Outside the repository: Hostinger's build log for test.gokesari.com is not visible from this run. Owner: hPanel → test.gokesari.com → Deployments → open the latest build log; then Redeploy → 'Settings and redeploy' (never 'Change repository'). A report-only merge to staging was also pushed to start a fresh build.</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Hostinger's SELLER_DATABASE_URL corrected; #218 makes migrateSplit refuse a seller URL that is not the core's linked seller database (clear message, nothing touched). test.gokesari.com built staging c2b1018 (#214 + #215 + #218) at 04:47 UTC on 20 Oct.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Fixed (#218)</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6986,8 +7038,96 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Staging (test.gokesari.com)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>After — run 1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Mobile (Lighthouse 12, simulated throttling)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>LCP 2.4 s, TBT 310 ms, CLS 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Staging (test.gokesari.com)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>After — run 2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Mobile (Lighthouse 12, simulated throttling)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>LCP 2.3 s, TBT 50 ms, CLS 0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6998,7 +7138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7587,12 +7727,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Staging not rebuilt after 55 min → recorded as a blocker; production held (release, production database migration and production tests not run).</t>
+          <t>Staging not rebuilt after 55 min → recorded as a blocker and production held until staging passed.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>The brief allows the next environment only after the previous one passes; the production database migration is held with the release so code and schema go together.</t>
+          <t>The brief allows the next environment only after the previous one passes.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7601,8 +7741,52 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Release checked against the two-database rules before it went further (owner request, 20 Oct): new tables classified (platform), migration tags (0086 core, 0087 seller), no seller↔customer foreign key, no writes to seller tables, no ON CONFLICT / session settings, the only transaction (banner order) touches core only with the audit after commit, no query joins seller and customer tables. CI test-split green on #214, #218 and the release.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE.md 'Two databases' rules.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>src/server/services/*; drizzle/0086, 0087; src/server/db/split/ownership.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>D-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Signed-in checks on staging not run: reading the sign-in code from the test accounts' mailbox (Gmail connector) to sign in was refused by this session's permission check; not worked around.</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Owner decides whether this run may sign in to the staging test accounts.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>tests/e2e/homepage-uiux.spec.ts ('signed in' group, local only)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D27"/>
+  <autoFilter ref="A1:D29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Homepage UI/UX: rollout state — staging live and tested, production not yet built (DEF-14)
Release #219 is on main (05:39 UTC) and the production databases have
0086–0087, but gokesari.com still serves a build without it at 06:49 UTC.
Recorded as DEF-14 (Hostinger build log needed); production tests run as
soon as the new home is live.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gs4EQHD7GwAULfSqxrdL9g
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GoKesari_Homepage_UIUX_Status_2026-10-20.xlsx
+++ b/docs/gokesari-audit/GoKesari_Homepage_UIUX_Status_2026-10-20.xlsx
@@ -17,11 +17,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Features'!$A$1:$K$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flows'!$A$1:$K$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Cases'!$A$1:$L$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Defects'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Defects'!$A$1:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lighthouse'!$A$1:$J$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$D$29</definedName>
   </definedNames>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>20 Oct 2026, 06:20 IST (00:50 UTC) — interim: staging not yet rebuilt by Hostinger (DEF-13); production held</t>
+          <t>20 Oct 2026, 12:20 IST (06:50 UTC) — staging deployed and tested; production released (#219) but not yet built by Hostinger (DEF-14)</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/sanjaymorankar-debug/GoKesari/pull/214 (feature) and https://github.com/sanjaymorankar-debug/GoKesari/pull/215 (split-site migration fix), branch claude/gifted-brahmagupta-nj0bt9 → staging (both merged)</t>
+          <t>Feature #214, fixes #215 / #218, release #219 (staging → main); results #217 (branch claude/gifted-brahmagupta-nj0bt9 → staging)</t>
         </is>
       </c>
     </row>
@@ -638,9 +638,9 @@
           <t>Playwright pass rate — Production</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
     </row>
@@ -887,23 +887,23 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Open blockers</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>3</v>
+          <t>Deploy — Production — site build</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Not live at 06:49 UTC: gokesari.com serves a build of 06:02 UTC without the release (DEF-14)</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>iOS native build: the 'iPhone app' workflow needs the repository secret EXPO_TOKEN and the Expo project id in mobile/app.config.ts (last run 18 Oct failed on both). Owner: add them (mobile/README.md 'iPhone builds from GitHub'), then Actions → iPhone app → Run (preview).</t>
-        </is>
+          <t>Open blockers</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -914,7 +914,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Android emulator / iOS simulator: this cloud environment has no Android SDK / KVM and no macOS. App checks ran as Playwright emulation of the app WebView (app user agent, touch, phone widths); the Android APKs are built by the 'Android APK' workflow on the PR.</t>
+          <t>Production deploy: gokesari.com has not built release #219 (DEF-14) — check the Hostinger build log for gokesari.com (most likely SELLER_DATABASE_URL, as on the test site) and redeploy. The production-safe suite, app checks and Lighthouse run as soon as the new home is live.</t>
         </is>
       </c>
     </row>
@@ -926,12 +926,36 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
+          <t>iOS native build: the 'iPhone app' workflow needs the repository secret EXPO_TOKEN and the Expo project id in mobile/app.config.ts (last run 18 Oct failed on both). Owner: add them (mobile/README.md 'iPhone builds from GitHub'), then Actions → iPhone app → Run (preview).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Android emulator / iOS simulator: this cloud environment has no Android SDK / KVM and no macOS. App checks ran as Playwright emulation of the app WebView (app user agent, touch, phone widths); the Android APKs are built by the 'Android APK' workflow on the PR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
           <t>Signed-in flows on staging / production: they need the emailed sign-in code of a test account. Reading it from the test mailbox was refused by this session's permission check (D-28); signed-in flows ran locally (F1-ACCOUNT-DESKTOP, F3-EMPTY-STATES, F6-FLOATING-CART, F2-RECENT-ACCOUNT, F1-BANNER-ADMIN). Staging sandbox payment (Cashfree) needs a signed-in session → not run in this pass.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B37"/>
+  <autoFilter ref="A1:B39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1051,9 +1075,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -1104,9 +1128,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -1161,9 +1185,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -1218,9 +1242,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -1271,9 +1295,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1324,9 +1348,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1381,9 +1405,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1438,9 +1462,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1491,9 +1515,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1544,9 +1568,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1597,9 +1621,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1650,9 +1674,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1707,9 +1731,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1760,9 +1784,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1813,9 +1837,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1866,9 +1890,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1919,9 +1943,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1972,9 +1996,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -2029,9 +2053,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -2082,9 +2106,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -2135,9 +2159,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -2188,9 +2212,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -2241,9 +2265,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2294,9 +2318,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2347,9 +2371,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -2404,9 +2428,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -2518,9 +2542,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2660,9 +2684,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -2713,9 +2737,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -2766,9 +2790,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -2819,9 +2843,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -2872,9 +2896,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2925,9 +2949,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -2978,9 +3002,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -3031,9 +3055,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -3084,9 +3108,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Waiting for the gokesari.com build</t>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Blocked (DEF-14)</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -6292,7 +6316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6783,8 +6807,40 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>DEF-14</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>gokesari.com has not deployed release #219 (merged 05:39 UTC) or #221 (06:15 UTC): at 06:49 UTC the site serves a build made at 06:02 UTC without the release (old home; /api/search/suggest and /admin/home-banners answer 404). The production databases already have 0086–0087 (run 39372089225) and are on the split layout.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Production (deploy)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Outside the repository: the Hostinger build log for gokesari.com is not visible from this run. Most likely the same cause as DEF-13 on the test site — the build's migration step (since #218) stops when SELLER_DATABASE_URL is not the seller database the core's foreign tables read (production: the database named PROD_SELLER_DATABASE_URL). Owner: hPanel → gokesari.com → Deployments → latest build log; fix SELLER_DATABASE_URL if the log says so, then Redeploy → 'Settings and redeploy'.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F15"/>
+  <autoFilter ref="A1:F16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Homepage UI/UX: production results and final status workbook (21 Oct)
gokesari.com built release #219 at 19:25 UTC on 20 Oct (DEF-14: a plain
Hostinger Redeploy rebuilt the last successful source, #216; a redeploy of
main fixed it). Production-safe guest suite (read-only): browser 30/30,
Android app emulation 20/20, iOS app emulation 22/22 cases;
batch-2026-10-remote + branding-footer 20/20; Lighthouse mobile 91 / 97
(was 84), accessibility 100. Final workbook GoKesari_Homepage_UIUX_Status_
2026-10-21.xlsx; DEF-15 records two production configuration items for the
owner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gs4EQHD7GwAULfSqxrdL9g
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GoKesari_Homepage_UIUX_Status_2026-10-20.xlsx
+++ b/docs/gokesari-audit/GoKesari_Homepage_UIUX_Status_2026-10-20.xlsx
@@ -17,12 +17,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Features'!$A$1:$K$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Flows'!$A$1:$K$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Test Cases'!$A$1:$L$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Defects'!$A$1:$F$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lighthouse'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Defects'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lighthouse'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Decisions'!$A$1:$D$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>20 Oct 2026, 12:20 IST (06:50 UTC) — staging deployed and tested; production released (#219) but not yet built by Hostinger (DEF-14)</t>
+          <t>21 Oct 2026, 06:25 IST (00:55 UTC) — final: local, staging and production pass; production tests read-only, no test data created</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Feature #214, fixes #215 / #218, release #219 (staging → main); results #217 (branch claude/gifted-brahmagupta-nj0bt9 → staging)</t>
+          <t>Feature #214, fixes #215 / #218, releases #219 / #221 (staging → main); results #217 (branch claude/gifted-brahmagupta-nj0bt9 → staging)</t>
         </is>
       </c>
     </row>
@@ -638,308 +638,308 @@
           <t>Playwright pass rate — Production</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>30/30 (100%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Playwright pass rate — Android</t>
+          <t xml:space="preserve">  run used for Production</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>20/20 (100%)</t>
+          <t>gokesari.com (https://gokesari.com, 2026-10-21T00:43)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  run used for Android</t>
+          <t>Playwright pass rate — Android</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>test.gokesari.com-app-android (https://test.gokesari.com, 2026-10-20T05:54)</t>
+          <t>20/20 (100%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Playwright pass rate — iOS</t>
+          <t xml:space="preserve">  run used for Android</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>22/22 (100%)</t>
+          <t>gokesari.com-app-android (https://gokesari.com, 2026-10-21T00:45)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  run used for iOS</t>
+          <t>Playwright pass rate — iOS</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>test.gokesari.com-app-ios (https://test.gokesari.com, 2026-10-20T05:56)</t>
+          <t>22/22 (100%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Unit + integration (Vitest, local, single DB)</t>
+          <t xml:space="preserve">  run used for iOS</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2,254 / 2,255 first run; the 1 failure (SEC-03) was a BOOTSTRAP_ADMIN_EMAILS value in the local .env; re-run of that file 28/28 → effectively 2,255 / 2,255</t>
+          <t>gokesari.com-app-ios (https://gokesari.com, 2026-10-21T00:48)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>New tests on the split layout (local)</t>
+          <t>Unit + integration (Vitest, local, single DB)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>39 / 39 (homepage-uiux unit + integration, price-comparison, db-split ownership); migrations 0086 → core, 0087 → seller applied on an existing split layout</t>
+          <t>2,254 / 2,255 first run; the 1 failure (SEC-03) was a BOOTSTRAP_ADMIN_EMAILS value in the local .env; re-run of that file 28/28 → effectively 2,255 / 2,255</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Mobile app (mobile/)</t>
+          <t>New tests on the split layout (local)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>typecheck ✓, lint ✓, 36 / 36 tests, Expo bundles Android + iOS ✓</t>
+          <t>39 / 39 (homepage-uiux unit + integration, price-comparison, db-split ownership); migrations 0086 → core, 0087 → seller applied on an existing split layout</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Lint / typecheck (web)</t>
+          <t>Mobile app (mobile/)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>0 errors (4 pre-existing warnings), tsc clean, production build ✓</t>
+          <t>typecheck ✓, lint ✓, 36 / 36 tests, Expo bundles Android + iOS ✓</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Android APK 1.3.0 (GitHub 'Android APK' workflow, PR #214)</t>
+          <t>Lint / typecheck (web)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Built ✓ — artifacts GoKesari-preview-apk and GoKesari-production-apk (run 39333658232, expire 18 Nov 2026)</t>
+          <t>0 errors (4 pre-existing warnings), tsc clean, production build ✓</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CI on PR #214</t>
+          <t>Android APK 1.3.0 (GitHub 'Android APK' workflow, PR #214)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>scope ✓, test ✓ (full suite), test-split ✓ (two-database layout), mobile ✓, APK preview ✓, APK production ✓ — merged into staging 19 Oct 22:49 UTC</t>
+          <t>Built ✓ — artifacts GoKesari-preview-apk and GoKesari-production-apk (run 39333658232, expire 18 Nov 2026)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Existing E2E regression (local)</t>
+          <t>CI on PR #214</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>acceptance 5/5 (sign-in, wallet top-up, subscribe 2 L/day, daily order + charge, change tomorrow, offline-only, access control, cron auth); mobile-app 5/7 (2 need the dev sign-in form, run on the dev server); branding-footer 8/8 (updated to the new footer); inventory-accounting, document-browser-read pass on the production build; regression-items-a-e 10 pass, then stops at the stale C1 step (Seller Central moved the shop contact card on 14 Oct — predates this change; later serial steps not reached, covered by integration tests)</t>
+          <t>scope ✓, test ✓ (full suite), test-split ✓ (two-database layout), mobile ✓, APK preview ✓, APK production ✓ — merged into staging 19 Oct 22:49 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Staging remote regression (batch-2026-10-remote + branding-footer)</t>
+          <t>Existing E2E regression (local)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>20 / 20 passed on test.gokesari.com (20 Oct 05:58 UTC)</t>
+          <t>acceptance 5/5 (sign-in, wallet top-up, subscribe 2 L/day, daily order + charge, change tomorrow, offline-only, access control, cron auth); mobile-app 5/7 (2 need the dev sign-in form, run on the dev server); branding-footer 8/8 (updated to the new footer); inventory-accounting, document-browser-read pass on the production build; regression-items-a-e 10 pass, then stops at the stale C1 step (Seller Central moved the shop contact card on 14 Oct — predates this change; later serial steps not reached, covered by integration tests)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — PR #214 merged</t>
+          <t>Staging remote regression (batch-2026-10-remote + branding-footer)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>19 Oct 2026 22:49 UTC (merge 1f4cd76)</t>
+          <t>20 / 20 passed on test.gokesari.com (20 Oct 05:58 UTC)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — fix PR #215 merged</t>
+          <t>Production remote regression (batch-2026-10-remote + branding-footer)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>19 Oct 2026 23:50 UTC (merge e6dab2d)</t>
+          <t>20 / 20 passed on gokesari.com (21 Oct 00:50 UTC), read-only</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging database (split: core + seller)</t>
+          <t>Android APK 1.3.0 — production build (main)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Test database run 39344001502, 23:51 UTC: backup ✓, 0086 → core, 0087 → seller, verify newest 0087 ✓</t>
+          <t>Built ✓ — Android APK workflow run 39376108294 on the release commit 80189e2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Staging — site build</t>
+          <t>Deploy — Staging — PR #214 merged</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>20 Oct 04:47 UTC: staging c2b1018 (#214 + #215 + #218) after Hostinger's SELLER_DATABASE_URL was corrected (DEF-13)</t>
+          <t>19 Oct 2026 22:49 UTC (merge 1f4cd76)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Split layout — staging</t>
+          <t>Deploy — Staging — fix PR #215 merged</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>split: core neondb, seller gokesari_seller (Database split switch-status, run 39376681434, 05:46 UTC)</t>
+          <t>19 Oct 2026 23:50 UTC (merge e6dab2d)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Split layout — production</t>
+          <t>Deploy — Staging database (split: core + seller)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>split: core neondb, seller PROD_SELLER_DATABASE_URL (Database split switch-status, run 39376683693, 05:46 UTC)</t>
+          <t>Test database run 39344001502, 23:51 UTC: backup ✓, 0086 → core, 0087 → seller, verify newest 0087 ✓</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Production database (0086, 0087)</t>
+          <t>Deploy — Staging — site build</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Production database run 39372089225, 04:55 UTC: restore point, migrate, state after ✓</t>
+          <t>20 Oct 04:47 UTC: staging c2b1018 (#214 + #215 + #218) after Hostinger's SELLER_DATABASE_URL was corrected (DEF-13)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Production — release #219 (staging → main)</t>
+          <t>Deploy — Split layout — staging</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>merged 20 Oct 05:39 UTC (80189e2), owner-approved</t>
+          <t>split: core neondb, seller gokesari_seller (Database split switch-status, run 39376681434, 05:46 UTC)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Deploy — Production — site build</t>
+          <t>Deploy — Split layout — production</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Not live at 06:49 UTC: gokesari.com serves a build of 06:02 UTC without the release (DEF-14)</t>
+          <t>split: core neondb, seller PROD_SELLER_DATABASE_URL (Database split switch-status, run 39376683693, 05:46 UTC)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Open blockers</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>5</v>
+          <t>Deploy — Production database (0086, 0087)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Production database run 39372089225, 04:55 UTC: restore point, migrate, state after ✓</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Production deploy: gokesari.com has not built release #219 (DEF-14) — check the Hostinger build log for gokesari.com (most likely SELLER_DATABASE_URL, as on the test site) and redeploy. The production-safe suite, app checks and Lighthouse run as soon as the new home is live.</t>
+          <t>Deploy — Production — release #219 (staging → main)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>merged 20 Oct 05:39 UTC (80189e2), owner-approved</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>iOS native build: the 'iPhone app' workflow needs the repository secret EXPO_TOKEN and the Expo project id in mobile/app.config.ts (last run 18 Oct failed on both). Owner: add them (mobile/README.md 'iPhone builds from GitHub'), then Actions → iPhone app → Run (preview).</t>
+          <t>Deploy — Production — site build</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Live 20 Oct 19:25 UTC (01:00 IST 21 Oct) after a redeploy of main (DEF-14); build uLTbrAiGsyctSEOjl_kyQ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Android emulator / iOS simulator: this cloud environment has no Android SDK / KVM and no macOS. App checks ran as Playwright emulation of the app WebView (app user agent, touch, phone widths); the Android APKs are built by the 'Android APK' workflow on the PR.</t>
-        </is>
+          <t>Open blockers</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -950,12 +950,36 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
+          <t>iOS native build: the 'iPhone app' workflow needs the repository secret EXPO_TOKEN and the Expo project id in mobile/app.config.ts (last run 18 Oct failed on both). Owner: add them (mobile/README.md 'iPhone builds from GitHub'), then Actions → iPhone app → Run (preview).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Android emulator / iOS simulator: this cloud environment has no Android SDK / KVM and no macOS. App checks ran as Playwright emulation of the app WebView (app user agent, touch, phone widths); the Android APKs are built by the 'Android APK' workflow on the PR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
           <t>Signed-in flows on staging / production: they need the emailed sign-in code of a test account. Reading it from the test mailbox was refused by this session's permission check (D-28); signed-in flows ran locally (F1-ACCOUNT-DESKTOP, F3-EMPTY-STATES, F6-FLOATING-CART, F2-RECENT-ACCOUNT, F1-BANNER-ADMIN). Staging sandbox payment (Cashfree) needs a signed-in session → not run in this pass.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B39"/>
+  <autoFilter ref="A1:B41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1075,9 +1099,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -1128,9 +1152,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -1185,9 +1209,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -1242,9 +1266,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -1295,9 +1319,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1348,9 +1372,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1405,9 +1429,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1462,9 +1486,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1515,9 +1539,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1568,9 +1592,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1621,9 +1645,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1674,9 +1698,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1731,9 +1755,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1784,9 +1808,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1837,9 +1861,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1890,9 +1914,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1943,9 +1967,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1996,9 +2020,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -2053,9 +2077,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -2106,9 +2130,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -2159,9 +2183,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -2212,9 +2236,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -2265,9 +2289,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2318,9 +2342,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -2371,9 +2395,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -2428,9 +2452,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -2542,9 +2566,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2684,9 +2708,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -2737,9 +2761,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -2790,9 +2814,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -2843,9 +2867,9 @@
           <t>Not run</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -2896,9 +2920,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2949,9 +2973,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -3002,9 +3026,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -3055,9 +3079,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -3108,9 +3132,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Blocked (DEF-14)</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -3958,7 +3982,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/APP-VOICE-1.2.0.png</t>
+          <t>iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/APP-VOICE-1.2.0.png</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4044,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/APP-VOICE-1.3.0.png</t>
+          <t>iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/APP-VOICE-1.3.0.png</t>
         </is>
       </c>
     </row>
@@ -4189,9 +4213,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -4208,8 +4232,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F1-DRAWER-GUEST.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F1-DRAWER-GUEST.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F1-DRAWER-GUEST.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F1-DRAWER-GUEST.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F1-DRAWER-GUEST.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F1-DRAWER-GUEST.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F1-DRAWER-GUEST.png</t>
         </is>
       </c>
     </row>
@@ -4254,9 +4279,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -4273,8 +4298,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F1-HERO.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F1-HERO.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F1-HERO.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F1-HERO.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F1-HERO.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F1-HERO.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F1-HERO.png</t>
         </is>
       </c>
     </row>
@@ -4319,9 +4345,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -4439,9 +4465,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -4458,8 +4484,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F2-SUGGEST-DESKTOP.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F2-SUGGEST-DESKTOP.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F2-SUGGEST-DESKTOP.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F2-SUGGEST-DESKTOP.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F2-SUGGEST-DESKTOP.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F2-SUGGEST-DESKTOP.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F2-SUGGEST-DESKTOP.png</t>
         </is>
       </c>
     </row>
@@ -4504,9 +4531,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -4523,8 +4550,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F2-VOICE.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F2-VOICE.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F2-VOICE.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F2-VOICE.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F2-VOICE.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F2-VOICE.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F2-VOICE.png</t>
         </is>
       </c>
     </row>
@@ -4631,9 +4659,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -4650,8 +4678,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F3-SEARCH-EMPTY.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F3-SEARCH-EMPTY.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F3-SEARCH-EMPTY.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F3-SEARCH-EMPTY.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F3-SEARCH-EMPTY.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F3-SEARCH-EMPTY.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F3-SEARCH-EMPTY.png</t>
         </is>
       </c>
     </row>
@@ -4696,9 +4725,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -4715,8 +4744,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F4-COMPARE.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F4-COMPARE.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F4-COMPARE.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F4-COMPARE.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F4-COMPARE.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F4-COMPARE.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F4-COMPARE.png</t>
         </is>
       </c>
     </row>
@@ -4761,9 +4791,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -4780,8 +4810,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F5-FOOTER.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F5-FOOTER.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F5-FOOTER.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F5-FOOTER.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F5-FOOTER.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F5-FOOTER.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F5-FOOTER.png</t>
         </is>
       </c>
     </row>
@@ -4888,9 +4919,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -4907,8 +4938,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F6-LOCATION-SHEET.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F6-LOCATION-SHEET.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F6-LOCATION-SHEET.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F6-LOCATION-SHEET.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F6-LOCATION-SHEET.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F6-LOCATION-SHEET.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F6-LOCATION-SHEET.png</t>
         </is>
       </c>
     </row>
@@ -4953,9 +4985,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -4972,8 +5004,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/F6-STICKY.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/F6-STICKY.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/F6-STICKY.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/F6-STICKY.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/F6-STICKY.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/F6-STICKY.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/F6-STICKY.png</t>
         </is>
       </c>
     </row>
@@ -5018,9 +5051,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -5036,7 +5069,8 @@
       <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-en.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-en.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-en.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-1024-en.png</t>
         </is>
       </c>
     </row>
@@ -5081,9 +5115,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -5099,7 +5133,8 @@
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-hi.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-hi.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-hi.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-1024-hi.png</t>
         </is>
       </c>
     </row>
@@ -5144,9 +5179,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -5162,7 +5197,8 @@
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1024-mr.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-mr.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1024-mr.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-1024-mr.png</t>
         </is>
       </c>
     </row>
@@ -5207,9 +5243,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -5225,7 +5261,8 @@
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-en.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-en.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-en.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-1440-en.png</t>
         </is>
       </c>
     </row>
@@ -5270,9 +5307,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -5288,7 +5325,8 @@
       <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-hi.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-hi.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-hi.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-1440-hi.png</t>
         </is>
       </c>
     </row>
@@ -5333,9 +5371,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -5351,7 +5389,8 @@
       <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-1440-mr.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-mr.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-1440-mr.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-1440-mr.png</t>
         </is>
       </c>
     </row>
@@ -5396,9 +5435,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -5415,8 +5454,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-360-en.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-360-en.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-360-en.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-360-en.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-360-en.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-360-en.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-360-en.png</t>
         </is>
       </c>
     </row>
@@ -5461,9 +5501,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -5480,8 +5520,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-360-hi.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-360-hi.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-360-hi.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-360-hi.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-360-hi.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-360-hi.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-360-hi.png</t>
         </is>
       </c>
     </row>
@@ -5526,9 +5567,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -5545,8 +5586,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-360-mr.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-360-mr.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-360-mr.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-360-mr.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-360-mr.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-360-mr.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-360-mr.png</t>
         </is>
       </c>
     </row>
@@ -5591,9 +5633,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -5610,8 +5652,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-390-en.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-390-en.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-390-en.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-390-en.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-390-en.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-390-en.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-390-en.png</t>
         </is>
       </c>
     </row>
@@ -5656,9 +5699,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -5675,8 +5718,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-390-hi.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-390-hi.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-390-hi.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-390-hi.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-390-hi.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-390-hi.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-390-hi.png</t>
         </is>
       </c>
     </row>
@@ -5721,9 +5765,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -5740,8 +5784,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-390-mr.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-390-mr.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-390-mr.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-390-mr.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-390-mr.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-390-mr.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-390-mr.png</t>
         </is>
       </c>
     </row>
@@ -5786,9 +5831,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -5805,8 +5850,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-414-en.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-414-en.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-414-en.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-414-en.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-414-en.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-414-en.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-414-en.png</t>
         </is>
       </c>
     </row>
@@ -5851,9 +5897,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -5870,8 +5916,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-414-hi.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-414-hi.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-414-hi.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-414-hi.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-414-hi.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-414-hi.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-414-hi.png</t>
         </is>
       </c>
     </row>
@@ -5916,9 +5963,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -5935,8 +5982,9 @@
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-414-mr.png
 Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-414-mr.png
-Android: e2e-evidence/homepage-uiux/test.gokesari.com-app-android/HP-414-mr.png
-iOS: e2e-evidence/homepage-uiux/test.gokesari.com-app-ios/HP-414-mr.png</t>
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-414-mr.png
+Android: e2e-evidence/homepage-uiux/gokesari.com-app-android/HP-414-mr.png
+iOS: e2e-evidence/homepage-uiux/gokesari.com-app-ios/HP-414-mr.png</t>
         </is>
       </c>
     </row>
@@ -5981,9 +6029,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
@@ -5999,7 +6047,8 @@
       <c r="L34" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-en.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-en.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-en.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-768-en.png</t>
         </is>
       </c>
     </row>
@@ -6044,9 +6093,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
@@ -6062,7 +6111,8 @@
       <c r="L35" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-hi.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-hi.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-hi.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-768-hi.png</t>
         </is>
       </c>
     </row>
@@ -6107,9 +6157,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -6125,7 +6175,8 @@
       <c r="L36" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/HP-768-mr.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-mr.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/HP-768-mr.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/HP-768-mr.png</t>
         </is>
       </c>
     </row>
@@ -6170,9 +6221,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -6228,9 +6279,9 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>Not run</t>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
@@ -6246,7 +6297,8 @@
       <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Local: e2e-evidence/homepage-uiux/localhost_3000/REG-SITE-HEADER.png
-Staging: e2e-evidence/homepage-uiux/test.gokesari.com/REG-SITE-HEADER.png</t>
+Staging: e2e-evidence/homepage-uiux/test.gokesari.com/REG-SITE-HEADER.png
+Production: e2e-evidence/homepage-uiux/gokesari.com/REG-SITE-HEADER.png</t>
         </is>
       </c>
     </row>
@@ -6316,7 +6368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6815,7 +6867,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>gokesari.com has not deployed release #219 (merged 05:39 UTC) or #221 (06:15 UTC): at 06:49 UTC the site serves a build made at 06:02 UTC without the release (old home; /api/search/suggest and /admin/home-banners answer 404). The production databases already have 0086–0087 (run 39372089225) and are on the split layout.</t>
+          <t>gokesari.com did not deploy release #219 (80189e2, merged 20 Oct 05:39 UTC) for ~14 h: it kept serving builds of #216 (6bb96c6). The owner's Hostinger log showed why redeploys never helped: a plain Redeploy restores the 'previous deployment source' (the last successful deployment, #216). Hostinger's variables were checked with the owner: DB_SPLIT_MODE=split and SELLER_DATABASE_URL opens PROD_SELLER_DATABASE_URL, the core's linked seller database, so the #218 seller check was not the cause.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -6830,17 +6882,49 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Outside the repository: the Hostinger build log for gokesari.com is not visible from this run. Most likely the same cause as DEF-13 on the test site — the build's migration step (since #218) stops when SELLER_DATABASE_URL is not the seller database the core's foreign tables read (production: the database named PROD_SELLER_DATABASE_URL). Owner: hPanel → gokesari.com → Deployments → latest build log; fix SELLER_DATABASE_URL if the log says so, then Redeploy → 'Settings and redeploy'.</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Redeployed from hPanel with the latest main; gokesari.com built the release at 19:25 UTC (20 Oct) and serves the new home, /api/search/suggest 200, /admin/home-banners → sign-in.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Fixed (redeploy of main)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>DEF-15</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Production configuration (seen while checking DEF-14, outside this change): INTEGRATION_ENCRYPTION_KEY on gokesari.com is not a 32-byte base64 key, so GSTIN linking fails and new bills are stored unencrypted (docs/inventory-accounting-2026-10/TESTING_REPORT.md). Production secrets (database password, AUTH_SECRET) were also shared in the session chat on 20 Oct.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Production (configuration)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Owner: set INTEGRATION_ENCRYPTION_KEY to the output of `openssl rand -base64 32` and redeploy; reset the neondb_owner password in Neon (update DATABASE_URL, SELLER_DATABASE_URL, PROD_* in Hostinger and the PROD_* GitHub secrets) and set a new AUTH_SECRET (signs everyone out once).</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Open (owner)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6851,7 +6935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7182,8 +7266,96 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Production (gokesari.com)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>After — run 1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Mobile (Lighthouse 12, simulated throttling)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>LCP 1.8 s, TBT 260 ms, CLS 0 (before: 84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Production (gokesari.com)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>After — run 2</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Mobile (Lighthouse 12, simulated throttling)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>LCP 1.8 s, TBT 80 ms, CLS 0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>